<commit_message>
Phase 3 (in progress): run log, run-close command, site data export, Vite site
Claude-Session: https://claude.ai/code/session_01QapJJnNjPZJPPwf6UNBBnr
</commit_message>
<xml_diff>
--- a/data/closes/2026-09-30/paquete_cierre_2026-09-30.xlsx
+++ b/data/closes/2026-09-30/paquete_cierre_2026-09-30.xlsx
@@ -520,7 +520,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Corte: 30/09/2026 23:59:59 hora de Buenos Aires. Cierre anterior: 30/06/2026. Generado: 2026-10-01T21:07:02+00:00 (UTC).</t>
+          <t>Corte: 30/09/2026 23:59:59 hora de Buenos Aires. Cierre anterior: 30/06/2026. Generado: 2026-10-01T22:04:51+00:00 (UTC).</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>rpc:mainnet.gateway.tenderly.co</t>
+          <t>blockscout:https://eth.blockscout.com/api</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>rpc:polygon.gateway.tenderly.co</t>
+          <t>blockscout:https://polygon.blockscout.com/api</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>rpc:worldchain-mainnet.gateway.tenderly.co</t>
+          <t>blockscout:https://worldchain-mainnet.explorer.alchemy.com/api</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1312,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>rpc:celo.gateway.tenderly.co</t>
+          <t>blockscout:https://celo.blockscout.com/api</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>rpc:mainnet.gateway.tenderly.co</t>
+          <t>blockscout:https://eth.blockscout.com/api</t>
         </is>
       </c>
     </row>
@@ -1554,7 +1554,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>rpc:polygon.gateway.tenderly.co</t>
+          <t>blockscout:https://polygon.blockscout.com/api</t>
         </is>
       </c>
     </row>
@@ -1698,7 +1698,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>rpc:worldchain-mainnet.gateway.tenderly.co</t>
+          <t>blockscout:https://worldchain-mainnet.explorer.alchemy.com/api</t>
         </is>
       </c>
     </row>
@@ -1746,7 +1746,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>rpc:celo.gateway.tenderly.co</t>
+          <t>blockscout:https://celo.blockscout.com/api</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>rpc:mainnet.gateway.tenderly.co</t>
+          <t>blockscout:https://eth.blockscout.com/api</t>
         </is>
       </c>
     </row>
@@ -1988,7 +1988,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>rpc:polygon.gateway.tenderly.co</t>
+          <t>blockscout:https://polygon.blockscout.com/api</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>rpc:worldchain-mainnet.gateway.tenderly.co</t>
+          <t>blockscout:https://worldchain-mainnet.explorer.alchemy.com/api</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2180,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>rpc:celo.gateway.tenderly.co</t>
+          <t>blockscout:https://celo.blockscout.com/api</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>rpc:mainnet.gateway.tenderly.co</t>
+          <t>blockscout:https://eth.blockscout.com/api</t>
         </is>
       </c>
     </row>
@@ -2422,7 +2422,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>rpc:polygon.gateway.tenderly.co</t>
+          <t>blockscout:https://polygon.blockscout.com/api</t>
         </is>
       </c>
     </row>
@@ -2566,7 +2566,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>rpc:worldchain-mainnet.gateway.tenderly.co</t>
+          <t>blockscout:https://worldchain-mainnet.explorer.alchemy.com/api</t>
         </is>
       </c>
     </row>
@@ -2614,7 +2614,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>rpc:celo.gateway.tenderly.co</t>
+          <t>blockscout:https://celo.blockscout.com/api</t>
         </is>
       </c>
     </row>
@@ -2760,7 +2760,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>rpc:mainnet.gateway.tenderly.co</t>
+          <t>blockscout:https://eth.blockscout.com/api</t>
         </is>
       </c>
     </row>
@@ -2856,7 +2856,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>rpc:polygon.gateway.tenderly.co</t>
+          <t>blockscout:https://polygon.blockscout.com/api</t>
         </is>
       </c>
     </row>
@@ -3000,7 +3000,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>rpc:worldchain-mainnet.gateway.tenderly.co</t>
+          <t>blockscout:https://worldchain-mainnet.explorer.alchemy.com/api</t>
         </is>
       </c>
     </row>
@@ -3048,7 +3048,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>rpc:celo.gateway.tenderly.co</t>
+          <t>blockscout:https://celo.blockscout.com/api</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>rpc:mainnet.gateway.tenderly.co</t>
+          <t>blockscout:https://eth.blockscout.com/api</t>
         </is>
       </c>
     </row>
@@ -3290,7 +3290,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>rpc:polygon.gateway.tenderly.co</t>
+          <t>blockscout:https://polygon.blockscout.com/api</t>
         </is>
       </c>
     </row>
@@ -3434,7 +3434,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>rpc:worldchain-mainnet.gateway.tenderly.co</t>
+          <t>blockscout:https://worldchain-mainnet.explorer.alchemy.com/api</t>
         </is>
       </c>
     </row>
@@ -3482,7 +3482,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>rpc:celo.gateway.tenderly.co</t>
+          <t>blockscout:https://celo.blockscout.com/api</t>
         </is>
       </c>
     </row>
@@ -13462,7 +13462,7 @@
       </c>
       <c r="M171" s="6" t="inlineStr">
         <is>
-          <t>Salió por el puente el 29/07/2026 hacia Celo y no encontramos la emisión del otro lado (buscada hasta el bloque 78988055 de Celo).</t>
+          <t>Salió por el puente el 29/07/2026 hacia Celo y no encontramos la emisión del otro lado (buscada hasta el bloque 78991528 de Celo).</t>
         </is>
       </c>
     </row>
@@ -20933,7 +20933,7 @@
       </c>
       <c r="M303" s="6" t="inlineStr">
         <is>
-          <t>Salió por el puente el 02/09/2026 hacia Gnosis y no encontramos la emisión del otro lado (buscada hasta el bloque 48539318 de Gnosis).</t>
+          <t>Salió por el puente el 02/09/2026 hacia Gnosis y no encontramos la emisión del otro lado (buscada hasta el bloque 48540003 de Gnosis).</t>
         </is>
       </c>
     </row>
@@ -30344,7 +30344,7 @@
       </c>
       <c r="M465" s="6" t="inlineStr">
         <is>
-          <t>Salió por el puente el 14/09/2026 hacia Ethereum y no encontramos la emisión del otro lado (buscada hasta el bloque 26100049 de Ethereum).</t>
+          <t>Salió por el puente el 14/09/2026 hacia Ethereum y no encontramos la emisión del otro lado (buscada hasta el bloque 26100337 de Ethereum).</t>
         </is>
       </c>
     </row>
@@ -41059,10 +41059,14 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
+          <t>blockscout:https://eth.blockscout.com/api</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>rpc:mainnet.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -41171,10 +41175,14 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
+          <t>blockscout:https://polygon.blockscout.com/api</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
           <t>rpc:polygon.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -41333,10 +41341,14 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
+          <t>blockscout:https://worldchain-mainnet.explorer.alchemy.com/api</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
           <t>rpc:worldchain-mainnet.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -41387,10 +41399,14 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
+          <t>blockscout:https://celo.blockscout.com/api</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
           <t>rpc:celo.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
@@ -41549,10 +41565,14 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
+          <t>blockscout:https://eth.blockscout.com/api</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
           <t>rpc:mainnet.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
@@ -41661,10 +41681,14 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
+          <t>blockscout:https://polygon.blockscout.com/api</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
           <t>rpc:polygon.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
@@ -41823,10 +41847,14 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
+          <t>blockscout:https://worldchain-mainnet.explorer.alchemy.com/api</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
           <t>rpc:worldchain-mainnet.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -41877,10 +41905,14 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
+          <t>blockscout:https://celo.blockscout.com/api</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
           <t>rpc:celo.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
@@ -42039,10 +42071,14 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
+          <t>blockscout:https://eth.blockscout.com/api</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
           <t>rpc:mainnet.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
@@ -42151,10 +42187,14 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
+          <t>blockscout:https://polygon.blockscout.com/api</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
           <t>rpc:polygon.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
@@ -42313,10 +42353,14 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
+          <t>blockscout:https://worldchain-mainnet.explorer.alchemy.com/api</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
           <t>rpc:worldchain-mainnet.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
@@ -42367,10 +42411,14 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
+          <t>blockscout:https://celo.blockscout.com/api</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
           <t>rpc:celo.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
@@ -42529,10 +42577,14 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
+          <t>blockscout:https://eth.blockscout.com/api</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
           <t>rpc:mainnet.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
@@ -42641,10 +42693,14 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
+          <t>blockscout:https://polygon.blockscout.com/api</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
           <t>rpc:polygon.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
@@ -42803,10 +42859,14 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
+          <t>blockscout:https://worldchain-mainnet.explorer.alchemy.com/api</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
           <t>rpc:worldchain-mainnet.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
     </row>
     <row r="35">
@@ -42857,10 +42917,14 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
+          <t>blockscout:https://celo.blockscout.com/api</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
           <t>rpc:celo.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
     </row>
     <row r="36">
@@ -43019,10 +43083,14 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
+          <t>blockscout:https://eth.blockscout.com/api</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
           <t>rpc:mainnet.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
     </row>
     <row r="39">
@@ -43131,10 +43199,14 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
+          <t>blockscout:https://polygon.blockscout.com/api</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
           <t>rpc:polygon.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
     </row>
     <row r="41">
@@ -43293,10 +43365,14 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
+          <t>blockscout:https://worldchain-mainnet.explorer.alchemy.com/api</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
           <t>rpc:worldchain-mainnet.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
     </row>
     <row r="44">
@@ -43347,10 +43423,14 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
+          <t>blockscout:https://celo.blockscout.com/api</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
           <t>rpc:celo.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
     </row>
     <row r="45">
@@ -43509,10 +43589,14 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
+          <t>blockscout:https://eth.blockscout.com/api</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
           <t>rpc:mainnet.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr"/>
     </row>
     <row r="48">
@@ -43621,10 +43705,14 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
+          <t>blockscout:https://polygon.blockscout.com/api</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
           <t>rpc:polygon.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr"/>
     </row>
     <row r="50">
@@ -43783,10 +43871,14 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
+          <t>blockscout:https://worldchain-mainnet.explorer.alchemy.com/api</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
           <t>rpc:worldchain-mainnet.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr"/>
     </row>
     <row r="53">
@@ -43837,10 +43929,14 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
+          <t>blockscout:https://celo.blockscout.com/api</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
           <t>rpc:celo.gateway.tenderly.co</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr"/>
     </row>
     <row r="54">

</xml_diff>

<commit_message>
Close run against the published site; tolerate plain-text RPC errors; keep failed engine output apart
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QapJJnNjPZJPPwf6UNBBnr
</commit_message>
<xml_diff>
--- a/data/closes/2026-09-30/paquete_cierre_2026-09-30.xlsx
+++ b/data/closes/2026-09-30/paquete_cierre_2026-09-30.xlsx
@@ -520,7 +520,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Corte: 30/09/2026 23:59:59 hora de Buenos Aires. Cierre anterior: 30/06/2026. Generado: 2026-10-01T22:04:51+00:00 (UTC).</t>
+          <t>Corte: 30/09/2026 23:59:59 hora de Buenos Aires. Cierre anterior: 30/06/2026. Generado: 2026-10-02T01:36:10+00:00 (UTC).</t>
         </is>
       </c>
     </row>
@@ -13462,7 +13462,7 @@
       </c>
       <c r="M171" s="6" t="inlineStr">
         <is>
-          <t>Salió por el puente el 29/07/2026 hacia Celo y no encontramos la emisión del otro lado (buscada hasta el bloque 78991528 de Celo).</t>
+          <t>Salió por el puente el 29/07/2026 hacia Celo y no encontramos la emisión del otro lado (buscada hasta el bloque 79004207 de Celo).</t>
         </is>
       </c>
     </row>
@@ -20933,7 +20933,7 @@
       </c>
       <c r="M303" s="6" t="inlineStr">
         <is>
-          <t>Salió por el puente el 02/09/2026 hacia Gnosis y no encontramos la emisión del otro lado (buscada hasta el bloque 48540003 de Gnosis).</t>
+          <t>Salió por el puente el 02/09/2026 hacia Gnosis y no encontramos la emisión del otro lado (buscada hasta el bloque 48542497 de Gnosis).</t>
         </is>
       </c>
     </row>
@@ -30344,7 +30344,7 @@
       </c>
       <c r="M465" s="6" t="inlineStr">
         <is>
-          <t>Salió por el puente el 14/09/2026 hacia Ethereum y no encontramos la emisión del otro lado (buscada hasta el bloque 26100337 de Ethereum).</t>
+          <t>Salió por el puente el 14/09/2026 hacia Ethereum y no encontramos la emisión del otro lado (buscada hasta el bloque 26101390 de Ethereum).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Exception agent: send the model decoded transaction fields only
get_transaction used to return raw topics and data prefixes for events it could not
decode, plus the full handleOps tuple signature. On World Chain (ERC-4337 handleOps)
that made the model's safeguards refuse step 2 almost every time, for Sonnet and the
Opus fallback alike. The result is now built by pure brief_transaction / brief_log:
function name, from, to, status, block and decoded events only (bridge events,
Minted, UserOperationEvent, RoleGranted, Approval, Transfer). contract_info no longer
returns the code hash. The code checks in exceptions.verify are unchanged.

Offline test with the recorded RPC answers of two refused cases. New close run:
2 refused calls instead of 7, both recovered on retry, 0 blocked cases instead of 3,
9 of 9 investigated, 4 resolved and 5 tasks, close figures unchanged.

Claude-Session: https://claude.ai/code/session_01QapJJnNjPZJPPwf6UNBBnr
</commit_message>
<xml_diff>
--- a/data/closes/2026-09-30/paquete_cierre_2026-09-30.xlsx
+++ b/data/closes/2026-09-30/paquete_cierre_2026-09-30.xlsx
@@ -520,7 +520,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Corte: 30/09/2026 23:59:59 hora de Buenos Aires. Cierre anterior: 30/06/2026. Generado: 2026-10-02T01:36:10+00:00 (UTC).</t>
+          <t>Corte: 30/09/2026 23:59:59 hora de Buenos Aires. Cierre anterior: 30/06/2026. Generado: 2026-10-02T02:10:35+00:00 (UTC).</t>
         </is>
       </c>
     </row>
@@ -13462,7 +13462,7 @@
       </c>
       <c r="M171" s="6" t="inlineStr">
         <is>
-          <t>Salió por el puente el 29/07/2026 hacia Celo y no encontramos la emisión del otro lado (buscada hasta el bloque 79004207 de Celo).</t>
+          <t>Salió por el puente el 29/07/2026 hacia Celo y no encontramos la emisión del otro lado (buscada hasta el bloque 79006268 de Celo).</t>
         </is>
       </c>
     </row>
@@ -20933,7 +20933,7 @@
       </c>
       <c r="M303" s="6" t="inlineStr">
         <is>
-          <t>Salió por el puente el 02/09/2026 hacia Gnosis y no encontramos la emisión del otro lado (buscada hasta el bloque 48542497 de Gnosis).</t>
+          <t>Salió por el puente el 02/09/2026 hacia Gnosis y no encontramos la emisión del otro lado (buscada hasta el bloque 48542905 de Gnosis).</t>
         </is>
       </c>
     </row>
@@ -30344,7 +30344,7 @@
       </c>
       <c r="M465" s="6" t="inlineStr">
         <is>
-          <t>Salió por el puente el 14/09/2026 hacia Ethereum y no encontramos la emisión del otro lado (buscada hasta el bloque 26101390 de Ethereum).</t>
+          <t>Salió por el puente el 14/09/2026 hacia Ethereum y no encontramos la emisión del otro lado (buscada hasta el bloque 26101562 de Ethereum).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verified means the two path check; second source becomes an extra check
- Verified: every pair reconciles by totalSupply at the cutoff block and by
  opening + mints - burns, exactly, and the method matches 9 of 9 certificates.
- Second source confirmation moves to a technical line in the Excel and on the
  page. Slack only flags a real discrepancy between two reconciling sources.
- Sources whose list does not reconcile are incomplete, not a discrepancy
  (Blockscout on Base).
- Etherscan "No records found" with an empty list is an empty range.
- 30/09 close regenerated with the free NodeReal and Etherscan keys: amounts,
  movements and the Slack message unchanged, 40 of 54 pairs confirmed by a
  second source.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MpyFq8aVkFbMHpvTMGAwCn
</commit_message>
<xml_diff>
--- a/data/closes/2026-09-30/paquete_cierre_2026-09-30.xlsx
+++ b/data/closes/2026-09-30/paquete_cierre_2026-09-30.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:L20"/>
+  <dimension ref="A2:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -520,7 +520,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Corte: 30/09/2026 23:59:59 hora de Buenos Aires. Cierre anterior: 30/06/2026. Generado: 2026-10-02T19:37:33+00:00 (UTC).</t>
+          <t>Corte: 30/09/2026 23:59:59 hora de Buenos Aires. Cierre anterior: 30/06/2026. Generado: 2026-10-03T18:09:23+00:00 (UTC).</t>
         </is>
       </c>
     </row>
@@ -531,6 +531,13 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Alcance: 54 de 54 pares token y red conciliados.</t>
+        </is>
+      </c>
+    </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
@@ -878,8 +885,22 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Verificado contra la blockchain: en cada red, la cantidad de tokens al corte coincide exacto, al último decimal, con la apertura más las emisiones menos las quemas.</t>
+        </is>
+      </c>
+    </row>
     <row r="20">
       <c r="A20" t="inlineStr">
+        <is>
+          <t>Control extra: una segunda fuente independiente confirmó cada movimiento en 40 de 54 pares. En el resto no hay una segunda fuente gratuita disponible y completa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Usa solo datos públicos: las blockchains y las certificaciones publicadas. No calcula el respaldo bancario.</t>
         </is>
@@ -1360,7 +1381,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>rpc:hyperliquid-json-rpc.stakely.io,rpc.hypurrscan.io</t>
+          <t>etherscan:https://api.etherscan.io/v2/api</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1815,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>rpc:hyperliquid-json-rpc.stakely.io,rpc.hypurrscan.io</t>
+          <t>etherscan:https://api.etherscan.io/v2/api</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2249,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>rpc:hyperliquid-json-rpc.stakely.io,rpc.hypurrscan.io</t>
+          <t>etherscan:https://api.etherscan.io/v2/api</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2683,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>rpc:hyperliquid-json-rpc.stakely.io,rpc.hypurrscan.io</t>
+          <t>etherscan:https://api.etherscan.io/v2/api</t>
         </is>
       </c>
     </row>
@@ -3096,7 +3117,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>rpc:hyperliquid-json-rpc.stakely.io,rpc.hypurrscan.io</t>
+          <t>etherscan:https://api.etherscan.io/v2/api</t>
         </is>
       </c>
     </row>
@@ -3530,7 +3551,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>rpc:hyperliquid-json-rpc.stakely.io,rpc.hypurrscan.io</t>
+          <t>etherscan:https://api.etherscan.io/v2/api</t>
         </is>
       </c>
     </row>
@@ -13462,7 +13483,7 @@
       </c>
       <c r="M171" s="6" t="inlineStr">
         <is>
-          <t>Salió por el puente el 29/07/2026 hacia Celo y no encontramos la emisión del otro lado (buscada hasta el bloque 79069091 de Celo).</t>
+          <t>Salió por el puente el 29/07/2026 hacia Celo y no encontramos la emisión del otro lado (buscada hasta el bloque 79150197 de Celo).</t>
         </is>
       </c>
     </row>
@@ -20933,7 +20954,7 @@
       </c>
       <c r="M303" s="6" t="inlineStr">
         <is>
-          <t>Salió por el puente el 02/09/2026 hacia Gnosis y no encontramos la emisión del otro lado (buscada hasta el bloque 48555205 de Gnosis).</t>
+          <t>Salió por el puente el 02/09/2026 hacia Gnosis y no encontramos la emisión del otro lado (buscada hasta el bloque 48571094 de Gnosis).</t>
         </is>
       </c>
     </row>
@@ -30344,7 +30365,7 @@
       </c>
       <c r="M465" s="6" t="inlineStr">
         <is>
-          <t>Salió por el puente el 14/09/2026 hacia Ethereum y no encontramos la emisión del otro lado (buscada hasta el bloque 26106772 de Ethereum).</t>
+          <t>Salió por el puente el 14/09/2026 hacia Ethereum y no encontramos la emisión del otro lado (buscada hasta el bloque 26113511 de Ethereum).</t>
         </is>
       </c>
     </row>
@@ -40933,7 +40954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:N57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -40948,6 +40969,8 @@
     <col width="40" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
     <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="60" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -41010,6 +41033,16 @@
           <t>Fuentes incompletas</t>
         </is>
       </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>Segunda fuente</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>Detalle de la segunda fuente</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -41068,6 +41101,16 @@
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Coinciden eth.blockscout.com y mainnet.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -41126,6 +41169,16 @@
           <t>blockscout:https://base.blockscout.com/api</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>una sola fuente</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Una sola fuente: base.blockscout.com devolvió una lista incompleta.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -41184,6 +41237,16 @@
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Coinciden polygon.blockscout.com y polygon.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -41238,6 +41301,16 @@
       </c>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>una sola fuente</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Una sola fuente: no hay una segunda fuente gratuita para esta red.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -41290,8 +41363,22 @@
           <t>bscscan list + RPC receipts</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>rpc:bsc-mainnet.nodereal.io/v1/***</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Coinciden bscscan list + RPC receipts y bsc-mainnet.nodereal.io.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -41350,6 +41437,16 @@
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Coinciden worldchain-mainnet.explorer.alchemy.com y worldchain-mainnet.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -41408,6 +41505,16 @@
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Coinciden celo.blockscout.com y celo.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -41457,11 +41564,25 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
+          <t>etherscan:https://api.etherscan.io/v2/api</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
           <t>rpc:hyperliquid-json-rpc.stakely.io,rpc.hypurrscan.io</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Coinciden api.etherscan.io y hyperliquid-json-rpc.stakely.io,rpc.hypurrscan.io.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -41516,6 +41637,16 @@
       </c>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>una sola fuente</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Una sola fuente: no hay una segunda fuente gratuita para esta red.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -41574,6 +41705,16 @@
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Coinciden eth.blockscout.com y mainnet.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -41632,6 +41773,16 @@
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Coinciden base.blockscout.com y mainnet.base.org.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -41690,6 +41841,16 @@
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Coinciden polygon.blockscout.com y polygon.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -41744,6 +41905,16 @@
       </c>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>una sola fuente</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Una sola fuente: no hay una segunda fuente gratuita para esta red.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -41796,8 +41967,22 @@
           <t>bscscan list + RPC receipts</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>rpc:bsc-mainnet.nodereal.io/v1/***</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Coinciden bscscan list + RPC receipts y bsc-mainnet.nodereal.io.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -41856,6 +42041,16 @@
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Coinciden worldchain-mainnet.explorer.alchemy.com y worldchain-mainnet.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -41914,6 +42109,16 @@
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Coinciden celo.blockscout.com y celo.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -41963,11 +42168,25 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
+          <t>etherscan:https://api.etherscan.io/v2/api</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
           <t>rpc:hyperliquid-json-rpc.stakely.io,rpc.hypurrscan.io</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Coinciden api.etherscan.io y hyperliquid-json-rpc.stakely.io,rpc.hypurrscan.io.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -42022,6 +42241,16 @@
       </c>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>una sola fuente</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Una sola fuente: no hay una segunda fuente gratuita para esta red.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -42080,6 +42309,16 @@
         </is>
       </c>
       <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Coinciden eth.blockscout.com y mainnet.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -42138,6 +42377,16 @@
         </is>
       </c>
       <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Coinciden base.blockscout.com y mainnet.base.org.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -42196,6 +42445,16 @@
         </is>
       </c>
       <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Coinciden polygon.blockscout.com y polygon.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -42250,6 +42509,16 @@
       </c>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>una sola fuente</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Una sola fuente: no hay una segunda fuente gratuita para esta red.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -42302,8 +42571,22 @@
           <t>bscscan list + RPC receipts</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>rpc:bsc-mainnet.nodereal.io/v1/***</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Coinciden bscscan list + RPC receipts y bsc-mainnet.nodereal.io.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -42362,6 +42645,16 @@
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Coinciden worldchain-mainnet.explorer.alchemy.com y worldchain-mainnet.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -42420,6 +42713,16 @@
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Coinciden celo.blockscout.com y celo.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -42469,11 +42772,25 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
+          <t>etherscan:https://api.etherscan.io/v2/api</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
           <t>rpc:hyperliquid-json-rpc.stakely.io,rpc.hypurrscan.io</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Coinciden api.etherscan.io y hyperliquid-json-rpc.stakely.io,rpc.hypurrscan.io.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -42528,6 +42845,16 @@
       </c>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>una sola fuente</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Una sola fuente: no hay una segunda fuente gratuita para esta red.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -42586,6 +42913,16 @@
         </is>
       </c>
       <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Coinciden eth.blockscout.com y mainnet.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -42644,6 +42981,16 @@
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Coinciden base.blockscout.com y mainnet.base.org.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -42702,6 +43049,16 @@
         </is>
       </c>
       <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Coinciden polygon.blockscout.com y polygon.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -42756,6 +43113,16 @@
       </c>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>una sola fuente</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Una sola fuente: no hay una segunda fuente gratuita para esta red.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -42808,8 +43175,22 @@
           <t>bscscan list + RPC receipts</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>rpc:bsc-mainnet.nodereal.io/v1/***</t>
+        </is>
+      </c>
       <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Coinciden bscscan list + RPC receipts y bsc-mainnet.nodereal.io.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -42868,6 +43249,16 @@
         </is>
       </c>
       <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Coinciden worldchain-mainnet.explorer.alchemy.com y worldchain-mainnet.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -42926,6 +43317,16 @@
         </is>
       </c>
       <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Coinciden celo.blockscout.com y celo.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -42975,11 +43376,25 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
+          <t>etherscan:https://api.etherscan.io/v2/api</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
           <t>rpc:hyperliquid-json-rpc.stakely.io,rpc.hypurrscan.io</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Coinciden api.etherscan.io y hyperliquid-json-rpc.stakely.io,rpc.hypurrscan.io.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -43034,6 +43449,16 @@
       </c>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>una sola fuente</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Una sola fuente: no hay una segunda fuente gratuita para esta red.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -43092,6 +43517,16 @@
         </is>
       </c>
       <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Coinciden eth.blockscout.com y mainnet.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -43150,6 +43585,16 @@
           <t>blockscout:https://base.blockscout.com/api</t>
         </is>
       </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>una sola fuente</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Una sola fuente: base.blockscout.com devolvió una lista incompleta.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -43208,6 +43653,16 @@
         </is>
       </c>
       <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Coinciden polygon.blockscout.com y polygon.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -43262,6 +43717,16 @@
       </c>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>una sola fuente</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Una sola fuente: no hay una segunda fuente gratuita para esta red.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -43314,8 +43779,22 @@
           <t>bscscan list + RPC receipts</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>rpc:bsc-mainnet.nodereal.io/v1/***</t>
+        </is>
+      </c>
       <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Coinciden bscscan list + RPC receipts y bsc-mainnet.nodereal.io.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -43374,6 +43853,16 @@
         </is>
       </c>
       <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Coinciden worldchain-mainnet.explorer.alchemy.com y worldchain-mainnet.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -43432,6 +43921,16 @@
         </is>
       </c>
       <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Coinciden celo.blockscout.com y celo.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -43481,11 +43980,25 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
+          <t>etherscan:https://api.etherscan.io/v2/api</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
           <t>rpc:hyperliquid-json-rpc.stakely.io,rpc.hypurrscan.io</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>Coinciden api.etherscan.io y hyperliquid-json-rpc.stakely.io,rpc.hypurrscan.io.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -43540,6 +44053,16 @@
       </c>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>una sola fuente</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Una sola fuente: no hay una segunda fuente gratuita para esta red.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -43598,6 +44121,16 @@
         </is>
       </c>
       <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Coinciden eth.blockscout.com y mainnet.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -43656,6 +44189,16 @@
         </is>
       </c>
       <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Coinciden base.blockscout.com y mainnet.base.org.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -43714,6 +44257,16 @@
         </is>
       </c>
       <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>Coinciden polygon.blockscout.com y polygon.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -43768,6 +44321,16 @@
       </c>
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>una sola fuente</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Una sola fuente: no hay una segunda fuente gratuita para esta red.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -43820,8 +44383,22 @@
           <t>bscscan list + RPC receipts</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>rpc:bsc-mainnet.nodereal.io/v1/***</t>
+        </is>
+      </c>
       <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>Coinciden bscscan list + RPC receipts y bsc-mainnet.nodereal.io.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -43880,6 +44457,16 @@
         </is>
       </c>
       <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Coinciden worldchain-mainnet.explorer.alchemy.com y worldchain-mainnet.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -43938,6 +44525,16 @@
         </is>
       </c>
       <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Coinciden celo.blockscout.com y celo.gateway.tenderly.co.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -43987,11 +44584,25 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
+          <t>etherscan:https://api.etherscan.io/v2/api</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
           <t>rpc:hyperliquid-json-rpc.stakely.io,rpc.hypurrscan.io</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>confirmado por una segunda fuente</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Coinciden api.etherscan.io y hyperliquid-json-rpc.stakely.io,rpc.hypurrscan.io.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -44046,6 +44657,16 @@
       </c>
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>una sola fuente</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Una sola fuente: no hay una segunda fuente gratuita para esta red.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">

</xml_diff>

<commit_message>
Classify direct mints by a token minter as primary issuance
A mint sent straight to the token contract by an account holding MINTER_ROLE
on the token at that block is primary issuance. The token is the transaction
target, so the caller of mint is proven. Mints through a wallet or another
contract stay unclassified for the exception agent.

This classifies the six February 2026 mints (H08) with onchain evidence and
no LLM call. The 2026-09-30 close keeps the same categories and amounts.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MpyFq8aVkFbMHpvTMGAwCn
</commit_message>
<xml_diff>
--- a/data/closes/2026-09-30/paquete_cierre_2026-09-30.xlsx
+++ b/data/closes/2026-09-30/paquete_cierre_2026-09-30.xlsx
@@ -520,7 +520,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Corte: 30/09/2026 23:59:59 hora de Buenos Aires. Cierre anterior: 30/06/2026. Generado: 2026-10-03T18:09:23+00:00 (UTC).</t>
+          <t>Corte: 30/09/2026 23:59:59 hora de Buenos Aires. Cierre anterior: 30/06/2026. Generado: 2026-10-03T18:32:34+00:00 (UTC).</t>
         </is>
       </c>
     </row>
@@ -13483,7 +13483,7 @@
       </c>
       <c r="M171" s="6" t="inlineStr">
         <is>
-          <t>Salió por el puente el 29/07/2026 hacia Celo y no encontramos la emisión del otro lado (buscada hasta el bloque 79150197 de Celo).</t>
+          <t>Salió por el puente el 29/07/2026 hacia Celo y no encontramos la emisión del otro lado (buscada hasta el bloque 79151590 de Celo).</t>
         </is>
       </c>
     </row>
@@ -20954,7 +20954,7 @@
       </c>
       <c r="M303" s="6" t="inlineStr">
         <is>
-          <t>Salió por el puente el 02/09/2026 hacia Gnosis y no encontramos la emisión del otro lado (buscada hasta el bloque 48571094 de Gnosis).</t>
+          <t>Salió por el puente el 02/09/2026 hacia Gnosis y no encontramos la emisión del otro lado (buscada hasta el bloque 48571369 de Gnosis).</t>
         </is>
       </c>
     </row>
@@ -30365,7 +30365,7 @@
       </c>
       <c r="M465" s="6" t="inlineStr">
         <is>
-          <t>Salió por el puente el 14/09/2026 hacia Ethereum y no encontramos la emisión del otro lado (buscada hasta el bloque 26113511 de Ethereum).</t>
+          <t>Salió por el puente el 14/09/2026 hacia Ethereum y no encontramos la emisión del otro lado (buscada hasta el bloque 26113625 de Ethereum).</t>
         </is>
       </c>
     </row>
@@ -44687,7 +44687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -44834,7 +44834,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Una quema es rescate primario si quien quema sus propios tokens tiene permiso de emisión (MINTER_ROLE) en el LimitedMinter de esa red, leído en el bloque de la quema.</t>
+          <t>Una emisión también es primaria si la transacción va directo al contrato del token y quien la envía tiene permiso de emisión (MINTER_ROLE) en el token, leído en el bloque de la emisión. Si pasa por una billetera u otro contrato, no se puede probar quién emitió y queda para el agente de excepciones.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -44844,14 +44844,14 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Lectura onchain de hasRole(MINTER_ROLE, cuenta) en el LimitedMinter verificado.</t>
+          <t>Lectura onchain de hasRole(MINTER_ROLE, cuenta) en el contrato del token (LatamStable).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Lo que no encaja en ninguna de estas reglas queda sin clasificar. No se adivina.</t>
+          <t>Una quema es rescate primario si quien quema sus propios tokens tiene permiso de emisión (MINTER_ROLE) en el LimitedMinter de esa red, leído en el bloque de la quema.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -44861,31 +44861,31 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Regla del motor.</t>
+          <t>Lectura onchain de hasRole(MINTER_ROLE, cuenta) en el LimitedMinter verificado.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>La cantidad en circulación es la suma de totalSupply() en las redes revisadas, sin excluir billeteras.</t>
+          <t>Lo que no encaja en ninguna de estas reglas queda sin clasificar. No se adivina.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>inferida</t>
+          <t>documentada</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Reproduce las 9 cifras certificadas publicadas (data/golden/verification.json).</t>
+          <t>Regla del motor.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>La comparación con las cifras certificadas se hace en tokens enteros.</t>
+          <t>La cantidad en circulación es la suma de totalSupply() en las redes revisadas, sin excluir billeteras.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -44895,14 +44895,14 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Regla única para las 9 certificaciones. Decisión de Máximo Sckell.</t>
+          <t>Reproduce las 9 cifras certificadas publicadas (data/golden/verification.json).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>El corte es a las 23:59:59 hora de Buenos Aires del último día del trimestre.</t>
+          <t>La comparación con las cifras certificadas se hace en tokens enteros.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -44912,39 +44912,56 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>En los cortes certificados, 23:59:59 de Buenos Aires y de UTC dan el mismo resultado.</t>
+          <t>Regla única para las 9 certificaciones. Decisión de Máximo Sckell.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Las redes revisadas son una lista escrita de redes EVM candidatas, cruzada con CoinGecko y con las redes que nombran los certificados.</t>
+          <t>El corte es a las 23:59:59 hora de Buenos Aires del último día del trimestre.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>documentada</t>
+          <t>inferida</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>config/chains.yaml, data/discovery.json y data/sources/coingecko_platforms.json.</t>
+          <t>En los cortes certificados, 23:59:59 de Buenos Aires y de UTC dan el mismo resultado.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
+          <t>Las redes revisadas son una lista escrita de redes EVM candidatas, cruzada con CoinGecko y con las redes que nombran los certificados.</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>documentada</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>config/chains.yaml, data/discovery.json y data/sources/coingecko_platforms.json.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
           <t>wUYU no se incluye: existe en las mismas redes, pero lo creó una fábrica pública y no hay evidencia de que sea de Ripio.</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>hipótesis</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>data/discovery.json</t>
         </is>

</xml_diff>